<commit_message>
Corrige quartas da Sul-Americana e atualiza artefatos
</commit_message>
<xml_diff>
--- a/sulamericana/datasets_sula/2_classificacao_por_jogo_quartas_sula.xlsx
+++ b/sulamericana/datasets_sula/2_classificacao_por_jogo_quartas_sula.xlsx
@@ -504,7 +504,7 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -536,7 +536,7 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -610,7 +610,7 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -642,7 +642,7 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -716,7 +716,7 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -822,7 +822,7 @@
         <v>0</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -854,7 +854,7 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>